<commit_message>
Making corrections to predictions!
</commit_message>
<xml_diff>
--- a/Benchmarks/Water Chemistry/Total Phosphorus/Var selection decisions 1-22-26.xlsx
+++ b/Benchmarks/Water Chemistry/Total Phosphorus/Var selection decisions 1-22-26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/adam_thompson_deq_oregon_gov/Documents/Documents/BioMonORDEQ/Benchmarks/Water Chemistry/Total Phosphorus/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/sabine_berzins_deq_oregon_gov/Documents/Documents/BioMonORDEQ/Benchmarks/Water Chemistry/Total Phosphorus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="264" documentId="8_{6B8D232A-EEA6-4563-A1A6-87C6EEBA49F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{101B7DC8-A99F-47D1-877F-3AD8987009FB}"/>
+  <xr:revisionPtr revIDLastSave="272" documentId="8_{6B8D232A-EEA6-4563-A1A6-87C6EEBA49F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1AC02D7-7984-4276-9ED4-557AE659CB7F}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1152" yWindow="1152" windowWidth="28500" windowHeight="14460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="234">
   <si>
     <t>num_vars</t>
   </si>
@@ -2847,7 +2847,7 @@
       <formula>NOT(ISERROR(SEARCH("REMOVE",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:C140" xr:uid="{EB42C186-6836-4773-A6E5-B88EA86420AD}">
       <formula1>"KEEP, REMOVE"</formula1>
     </dataValidation>
@@ -2858,365 +2858,582 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{077211B4-8B56-4334-A6B9-B5C347A0B98D}">
-  <dimension ref="A1:A75"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E22" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E25" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E26" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E27" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E30" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E31" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E35" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E36" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E38" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E39" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E40" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E41" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E42" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E43" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E44" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E45" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E46" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E47" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E48" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E49" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E50" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E51" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E52" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E53" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E54" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E55" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E56" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E57" t="s">
+        <v>109</v>
+      </c>
+      <c r="I57" t="str">
+        <f>_xlfn.TEXTJOIN(", ", TRUE, E1:E71)</f>
+        <v>BFIWS, CANALDENSWS, CLAYWS, COMPSTRGTHWS, DAMNRMSTORWS, ELEVWS, FE2O3WS, FERTWS, HYDRLCONDWS, INORGNWETDEP2008WS, K2OWS, KFFACTWS, MINEDENSWS, MSST2008, NANIWS, NHD_pSLOPE, NPDESDENSWS, NWS, OMWS, P2O5WS, PCT_EROD, PCTAGDRAINAGEWS, PCTALKINTRUVOLWS, PCTALLUVCOASTWS, PCTBL2001WS, PCTBURNAREA2002WS, PCTCARBRESIDWS, PCTCOLLUVSEDWS, PCTCONIF2001WS, PCTCROP2001WS, PCTDECID2001WS, PCTEOLFINEWS, PCTEXTRUVOLWS, PCTFRSTLOSS2002WS, PCTGLACLAKECRSWS, PCTGLACLAKEFINEWS, PCTGLACTILCRSWS, PCTGRS2001WS, PCTHAY2001WS, PCTHBWET2001WS, PCTICE2001WS, PCTIMP2001WS, PCTINCVEGRESP2002WS, PCTNONAGINTRODMANAGVEGWS, PCTOW2001WS, PCTSALLAKEWS, PCTSHRB2001WS, PCTURBHI2001WS, PCTURBLO2001WS, PCTURBOP2001WS, PCTWATERWS, PCTWDWET2001WS, PESTIC1997WS, POPDEN2010WS, RCKDEPWS, RDCRSSLPWTDWS, RDCRSWS, RDDENSWS, ROCKNWS, SANDWS, SEPTICWS, STRMPOW_CAT, SUPERFUNDDENSWS, SW_FLUXWS, SWS, TMAX9120WS, TRIDENSWS, WETINDEXWS, WTDEPWS, WWTPALLDENSWS, WWTPMAJORDENSWS</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E58" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E59" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E60" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E61" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E62" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E63" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E64" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E65" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E66" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E67" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E68" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E69" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E70" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="E71" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="str">
         <f>_xlfn.TEXTJOIN(", ", TRUE, A1:A71)</f>
         <v>BFIWS, CANALDENSWS, CLAYWS, COMPSTRGTHWS, DAMNRMSTORWS, ELEVWS, FE2O3WS, FERTWS, HYDRLCONDWS, K2OWS, KFFACTWS, MINEDENSWS, MSST2008, NANIWS, NHD_pSLOPE, NPDESDENSWS, NWS, OMWS, P2O5WS, PCT_EROD, PCTAGDRAINAGEWS, PCTALKINTRUVOLWS, PCTALLUVCOASTWS, PCTBL2001WS, PCTBURNAREA2002WS, PCTCARBRESIDWS, PCTCOLLUVSEDWS, PCTCONIF2001WS, PCTCROP2001WS, PCTDECID2001WS, PCTEOLFINEWS, PCTEXTRUVOLWS, PCTFRSTLOSS2002WS, PCTGLACLAKECRSWS, PCTGLACLAKEFINEWS, PCTGLACTILCRSWS, PCTGRS2001WS, PCTHAY2001WS, PCTHBWET2001WS, PCTICE2001WS, PCTIMP2001WS, PCTINCVEGRESP2002WS, PCTNONAGINTRODMANAGVEGWS, PCTOW2001WS, PCTSALLAKEWS, PCTSHRB2001WS, PCTURBHI2001WS, PCTURBLO2001WS, PCTURBOP2001WS, PCTWATERWS, PCTWDWET2001WS, PESTIC1997WS, POPDEN2010WS, PRECIP_MINUS_EVTWS, RCKDEPWS, RDCRSSLPWTDWS, RDCRSWS, RDDENSWS, ROCKNWS, SANDWS, SEPTICWS, STRMPOW_CAT, SUPERFUNDDENSWS, SW_FLUXWS, SWS, TMAX9120WS, TRIDENSWS, WETINDEXWS, WTDEPWS, WWTPALLDENSWS, WWTPMAJORDENSWS</v>

</xml_diff>